<commit_message>
Canonicalize final D1-D5 quality dimensions
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D1 Sensor health/outputs/data/D1_recovery_validation.xlsx
+++ b/Project 1 Data Quality Assessment/D1 Sensor health/outputs/data/D1_recovery_validation.xlsx
@@ -662,7 +662,7 @@
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
@@ -759,7 +759,7 @@
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
@@ -856,7 +856,7 @@
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr">
@@ -953,7 +953,7 @@
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr">
@@ -3326,7 +3326,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -3381,7 +3381,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -3434,7 +3434,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -3542,7 +3542,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -3650,7 +3650,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -3703,7 +3703,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -3813,7 +3813,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -3868,7 +3868,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -3921,7 +3921,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -3976,7 +3976,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -4031,7 +4031,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -4086,7 +4086,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -4139,7 +4139,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -4194,7 +4194,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -4249,7 +4249,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -4302,7 +4302,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -4355,7 +4355,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -4410,7 +4410,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -4465,7 +4465,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -4518,7 +4518,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -4571,7 +4571,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -4626,7 +4626,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -4681,7 +4681,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -4736,7 +4736,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -4789,7 +4789,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -4844,7 +4844,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -4899,7 +4899,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -5007,7 +5007,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -5062,7 +5062,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -5117,7 +5117,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -5170,7 +5170,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -5223,7 +5223,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -5278,7 +5278,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -5333,7 +5333,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -5386,7 +5386,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -5439,7 +5439,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -5494,7 +5494,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -5549,7 +5549,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -5604,7 +5604,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -5657,7 +5657,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -5712,7 +5712,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -5767,7 +5767,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -5822,7 +5822,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5875,7 +5875,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -5930,7 +5930,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -5985,7 +5985,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -6038,7 +6038,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -6091,7 +6091,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -6146,7 +6146,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6201,7 +6201,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -6254,7 +6254,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -6307,7 +6307,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -6417,7 +6417,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -6472,7 +6472,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -6525,7 +6525,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -6580,7 +6580,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -6635,7 +6635,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -6690,7 +6690,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -6743,7 +6743,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -6798,7 +6798,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -6853,7 +6853,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -6906,7 +6906,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -6959,7 +6959,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -7069,7 +7069,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -7122,7 +7122,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -7175,7 +7175,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -7230,7 +7230,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -7285,7 +7285,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -7340,7 +7340,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -7393,7 +7393,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -7448,7 +7448,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -7503,7 +7503,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -7558,7 +7558,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -7611,7 +7611,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -7666,7 +7666,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -7721,7 +7721,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -7774,7 +7774,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -7882,7 +7882,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -7937,7 +7937,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -7990,7 +7990,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -8043,7 +8043,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -8098,7 +8098,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -8153,7 +8153,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -8208,7 +8208,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -8261,7 +8261,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -8316,7 +8316,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -8371,7 +8371,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -8426,7 +8426,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -8479,7 +8479,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -8534,7 +8534,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -8589,7 +8589,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -8642,7 +8642,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -8695,7 +8695,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -8750,7 +8750,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -8805,7 +8805,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -8858,7 +8858,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -8911,7 +8911,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -8966,7 +8966,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -9021,7 +9021,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -9076,7 +9076,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -9129,7 +9129,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -9184,7 +9184,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -9239,7 +9239,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -9294,7 +9294,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -9347,7 +9347,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -9402,7 +9402,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -9457,7 +9457,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -9510,7 +9510,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -9563,7 +9563,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -9618,7 +9618,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -9673,7 +9673,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -9726,7 +9726,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -9779,7 +9779,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -9834,7 +9834,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -9889,7 +9889,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -9944,7 +9944,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -9997,7 +9997,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -10052,7 +10052,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -10107,7 +10107,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -10162,7 +10162,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -10215,7 +10215,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -10270,7 +10270,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -10325,7 +10325,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -10378,7 +10378,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -10431,7 +10431,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -10486,7 +10486,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -10541,7 +10541,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -10594,7 +10594,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -10647,7 +10647,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -10702,7 +10702,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -10757,7 +10757,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -10812,7 +10812,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -10865,7 +10865,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -10920,7 +10920,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -10975,7 +10975,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -11030,7 +11030,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -11083,7 +11083,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -11138,7 +11138,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -11193,7 +11193,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -11246,7 +11246,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -11299,7 +11299,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -11354,7 +11354,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -11409,7 +11409,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -11462,7 +11462,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -11515,7 +11515,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -11570,7 +11570,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -11625,7 +11625,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -11680,7 +11680,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -11733,7 +11733,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -11788,7 +11788,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -11843,7 +11843,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -11898,7 +11898,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -11951,7 +11951,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -12006,7 +12006,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -12061,7 +12061,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -12114,7 +12114,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -12167,7 +12167,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -12222,7 +12222,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -12277,7 +12277,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -12330,7 +12330,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -12383,7 +12383,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -12438,7 +12438,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -12493,7 +12493,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -12548,7 +12548,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -12601,7 +12601,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -12656,7 +12656,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -12711,7 +12711,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -12766,7 +12766,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -12819,7 +12819,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -12874,7 +12874,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -12929,7 +12929,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -12982,7 +12982,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -13035,7 +13035,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -13090,7 +13090,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -13145,7 +13145,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -13198,7 +13198,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -13251,7 +13251,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -13306,7 +13306,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -13361,7 +13361,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -13416,7 +13416,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -13469,7 +13469,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
@@ -13524,7 +13524,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
@@ -13579,7 +13579,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -13634,7 +13634,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -13687,7 +13687,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -13742,7 +13742,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -13797,7 +13797,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -13850,7 +13850,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -13903,7 +13903,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
@@ -13958,7 +13958,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -14013,7 +14013,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
@@ -14066,7 +14066,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -14119,7 +14119,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
@@ -14174,7 +14174,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
@@ -14229,7 +14229,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
@@ -14284,7 +14284,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
@@ -14337,7 +14337,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
@@ -14392,7 +14392,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
@@ -14447,7 +14447,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
@@ -14502,7 +14502,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
@@ -14555,7 +14555,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
@@ -14610,7 +14610,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
@@ -14665,7 +14665,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
@@ -14718,7 +14718,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
@@ -14771,7 +14771,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
@@ -14826,7 +14826,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
@@ -14881,7 +14881,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
@@ -14934,7 +14934,7 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
@@ -14987,7 +14987,7 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
@@ -15042,7 +15042,7 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
@@ -15097,7 +15097,7 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
@@ -15152,7 +15152,7 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
@@ -15205,7 +15205,7 @@
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D221" t="inlineStr">
@@ -15260,7 +15260,7 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D222" t="inlineStr">
@@ -15315,7 +15315,7 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
@@ -15370,7 +15370,7 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D224" t="inlineStr">
@@ -15423,7 +15423,7 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D225" t="inlineStr">
@@ -16132,7 +16132,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -16276,7 +16276,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -16420,7 +16420,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -16564,7 +16564,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -16746,7 +16746,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>d1-final-ab36d51d4f60</t>
+          <t>d1-final-33fa914b2f71</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>